<commit_message>
Added fertilizer schedules for four years
</commit_message>
<xml_diff>
--- a/Data/2007_F111_CO_ISM/2007_F111_CO_ISM_Management.xlsx
+++ b/Data/2007_F111_CO_ISM/2007_F111_CO_ISM_Management.xlsx
@@ -1,21 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mnt\Data1\USDA-ALARC\GIS\PDI project\cottondata\Data\2007_F111_CO_ISM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3C0A1F2-1386-4CFF-8297-B348F0FF6B03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B555EA4D-350A-4417-8E29-882206A2A58E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16335" yWindow="-18195" windowWidth="17850" windowHeight="16440" xr2:uid="{118525E0-BC31-4C3F-8132-452FA3C5B73C}"/>
+    <workbookView xWindow="16470" yWindow="-25965" windowWidth="17865" windowHeight="22530" activeTab="4" xr2:uid="{118525E0-BC31-4C3F-8132-452FA3C5B73C}"/>
   </bookViews>
   <sheets>
     <sheet name="Irrigation" sheetId="3" r:id="rId1"/>
     <sheet name="Timeline" sheetId="2" r:id="rId2"/>
     <sheet name="IrrigationDF" sheetId="1" r:id="rId3"/>
+    <sheet name="Fertilizer" sheetId="4" r:id="rId4"/>
+    <sheet name="FertilizerDF" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="90">
   <si>
     <t>Year</t>
   </si>
@@ -405,14 +407,18 @@
   <si>
     <t>p08</t>
   </si>
+  <si>
+    <t>Convert lb/ac to kg/ha</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="[$-409]d\-mmm\-yy;@"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -740,7 +746,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -766,10 +772,16 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="260">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4565,163 +4577,163 @@
         <v>2</v>
       </c>
       <c r="E53" s="4">
-        <f>SUM(E7:E50)</f>
+        <f t="shared" ref="E53:AR53" si="0">SUM(E7:E50)</f>
         <v>890</v>
       </c>
       <c r="F53" s="4">
-        <f>SUM(F7:F50)</f>
+        <f t="shared" si="0"/>
         <v>778</v>
       </c>
       <c r="G53" s="4">
-        <f>SUM(G7:G50)</f>
+        <f t="shared" si="0"/>
         <v>926</v>
       </c>
       <c r="H53" s="4">
-        <f>SUM(H7:H50)</f>
+        <f t="shared" si="0"/>
         <v>912</v>
       </c>
       <c r="I53" s="4">
-        <f>SUM(I7:I50)</f>
+        <f t="shared" si="0"/>
         <v>886</v>
       </c>
       <c r="J53" s="4">
-        <f>SUM(J7:J50)</f>
+        <f t="shared" si="0"/>
         <v>906</v>
       </c>
       <c r="K53" s="4">
-        <f>SUM(K7:K50)</f>
+        <f t="shared" si="0"/>
         <v>806</v>
       </c>
       <c r="L53" s="4">
-        <f>SUM(L7:L50)</f>
+        <f t="shared" si="0"/>
         <v>797</v>
       </c>
       <c r="M53" s="4">
-        <f>SUM(M7:M50)</f>
+        <f t="shared" si="0"/>
         <v>889</v>
       </c>
       <c r="N53" s="4">
-        <f>SUM(N7:N50)</f>
+        <f t="shared" si="0"/>
         <v>808</v>
       </c>
       <c r="O53" s="4">
-        <f>SUM(O7:O50)</f>
+        <f t="shared" si="0"/>
         <v>915</v>
       </c>
       <c r="P53" s="4">
-        <f>SUM(P7:P50)</f>
+        <f t="shared" si="0"/>
         <v>812</v>
       </c>
       <c r="Q53" s="4">
-        <f>SUM(Q7:Q50)</f>
+        <f t="shared" si="0"/>
         <v>941</v>
       </c>
       <c r="R53" s="4">
-        <f>SUM(R7:R50)</f>
+        <f t="shared" si="0"/>
         <v>841</v>
       </c>
       <c r="S53" s="4">
-        <f>SUM(S7:S50)</f>
+        <f t="shared" si="0"/>
         <v>936</v>
       </c>
       <c r="T53" s="4">
-        <f>SUM(T7:T50)</f>
+        <f t="shared" si="0"/>
         <v>931</v>
       </c>
       <c r="U53" s="4">
-        <f>SUM(U7:U50)</f>
+        <f t="shared" si="0"/>
         <v>879</v>
       </c>
       <c r="V53" s="4">
-        <f>SUM(V7:V50)</f>
+        <f t="shared" si="0"/>
         <v>909</v>
       </c>
       <c r="W53" s="4">
-        <f>SUM(W7:W50)</f>
+        <f t="shared" si="0"/>
         <v>893</v>
       </c>
       <c r="X53" s="4">
-        <f>SUM(X7:X50)</f>
+        <f t="shared" si="0"/>
         <v>784</v>
       </c>
       <c r="Y53" s="4">
-        <f>SUM(Y7:Y50)</f>
+        <f t="shared" si="0"/>
         <v>900</v>
       </c>
       <c r="Z53" s="4">
-        <f>SUM(Z7:Z50)</f>
+        <f t="shared" si="0"/>
         <v>792</v>
       </c>
       <c r="AA53" s="4">
-        <f>SUM(AA7:AA50)</f>
+        <f t="shared" si="0"/>
         <v>826</v>
       </c>
       <c r="AB53" s="4">
-        <f>SUM(AB7:AB50)</f>
+        <f t="shared" si="0"/>
         <v>799</v>
       </c>
       <c r="AC53" s="4">
-        <f>SUM(AC7:AC50)</f>
+        <f t="shared" si="0"/>
         <v>795</v>
       </c>
       <c r="AD53" s="4">
-        <f>SUM(AD7:AD50)</f>
+        <f t="shared" si="0"/>
         <v>776</v>
       </c>
       <c r="AE53" s="4">
-        <f>SUM(AE7:AE50)</f>
+        <f t="shared" si="0"/>
         <v>840</v>
       </c>
       <c r="AF53" s="4">
-        <f>SUM(AF7:AF50)</f>
+        <f t="shared" si="0"/>
         <v>926</v>
       </c>
       <c r="AG53" s="4">
-        <f>SUM(AG7:AG50)</f>
+        <f t="shared" si="0"/>
         <v>884</v>
       </c>
       <c r="AH53" s="4">
-        <f>SUM(AH7:AH50)</f>
+        <f t="shared" si="0"/>
         <v>907</v>
       </c>
       <c r="AI53" s="4">
-        <f>SUM(AI7:AI50)</f>
+        <f t="shared" si="0"/>
         <v>833</v>
       </c>
       <c r="AJ53" s="4">
-        <f>SUM(AJ7:AJ50)</f>
+        <f t="shared" si="0"/>
         <v>886</v>
       </c>
       <c r="AK53" s="4">
-        <f>SUM(AK7:AK50)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AL53" s="4">
-        <f>SUM(AL7:AL50)</f>
+        <f t="shared" si="0"/>
         <v>856</v>
       </c>
       <c r="AM53" s="4">
-        <f>SUM(AM7:AM50)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AN53" s="4">
-        <f>SUM(AN7:AN50)</f>
+        <f t="shared" si="0"/>
         <v>837</v>
       </c>
       <c r="AO53" s="4">
-        <f>SUM(AO7:AO50)</f>
+        <f t="shared" si="0"/>
         <v>833</v>
       </c>
       <c r="AP53" s="4">
-        <f>SUM(AP7:AP50)</f>
+        <f t="shared" si="0"/>
         <v>861</v>
       </c>
       <c r="AQ53" s="4">
-        <f>SUM(AQ7:AQ50)</f>
+        <f t="shared" si="0"/>
         <v>840</v>
       </c>
       <c r="AR53" s="4">
-        <f>SUM(AR7:AR50)</f>
+        <f t="shared" si="0"/>
         <v>821</v>
       </c>
     </row>
@@ -4733,55 +4745,55 @@
     </row>
     <row r="56" spans="1:45" x14ac:dyDescent="0.2">
       <c r="AF56" s="4">
-        <f>SUM(AF10:AF53)</f>
+        <f t="shared" ref="AF56:AR56" si="1">SUM(AF10:AF53)</f>
         <v>1717</v>
       </c>
       <c r="AG56" s="4">
-        <f>SUM(AG10:AG53)</f>
+        <f t="shared" si="1"/>
         <v>1644</v>
       </c>
       <c r="AH56" s="4">
-        <f>SUM(AH10:AH53)</f>
+        <f t="shared" si="1"/>
         <v>1674</v>
       </c>
       <c r="AI56" s="4">
-        <f>SUM(AI10:AI53)</f>
+        <f t="shared" si="1"/>
         <v>1522</v>
       </c>
       <c r="AJ56" s="4">
-        <f>SUM(AJ10:AJ53)</f>
+        <f t="shared" si="1"/>
         <v>1631</v>
       </c>
       <c r="AK56" s="4">
-        <f>SUM(AK10:AK53)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AL56" s="4">
-        <f>SUM(AL10:AL53)</f>
+        <f t="shared" si="1"/>
         <v>1560</v>
       </c>
       <c r="AM56" s="4">
-        <f>SUM(AM10:AM53)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AN56" s="4">
-        <f>SUM(AN10:AN53)</f>
+        <f t="shared" si="1"/>
         <v>1522</v>
       </c>
       <c r="AO56" s="4">
-        <f>SUM(AO10:AO53)</f>
+        <f t="shared" si="1"/>
         <v>1514</v>
       </c>
       <c r="AP56" s="4">
-        <f>SUM(AP10:AP53)</f>
+        <f t="shared" si="1"/>
         <v>1563</v>
       </c>
       <c r="AQ56" s="4">
-        <f>SUM(AQ10:AQ53)</f>
+        <f t="shared" si="1"/>
         <v>1533</v>
       </c>
       <c r="AR56" s="4">
-        <f>SUM(AR10:AR53)</f>
+        <f t="shared" si="1"/>
         <v>1499</v>
       </c>
       <c r="AS56" s="4">
@@ -5225,135 +5237,132 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{308C26F9-EBC4-44FF-A8C7-3B54AE702DF4}">
   <dimension ref="A1:AP34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="9.140625" style="17"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:42" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="F1" s="18" t="s">
+      <c r="F1" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="G1" s="18" t="s">
+      <c r="G1" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="H1" s="18" t="s">
+      <c r="H1" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="I1" s="18" t="s">
+      <c r="I1" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="J1" s="18" t="s">
+      <c r="J1" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="K1" s="18" t="s">
+      <c r="K1" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="L1" s="18" t="s">
+      <c r="L1" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="M1" s="18" t="s">
+      <c r="M1" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="N1" s="18" t="s">
+      <c r="N1" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="O1" s="18" t="s">
+      <c r="O1" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="P1" s="18" t="s">
+      <c r="P1" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="Q1" s="18" t="s">
+      <c r="Q1" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="R1" s="18" t="s">
+      <c r="R1" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="S1" s="18" t="s">
+      <c r="S1" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="T1" s="18" t="s">
+      <c r="T1" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="U1" s="18" t="s">
+      <c r="U1" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="V1" s="18" t="s">
+      <c r="V1" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="W1" s="18" t="s">
+      <c r="W1" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="X1" s="18" t="s">
+      <c r="X1" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="Y1" s="18" t="s">
+      <c r="Y1" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="Z1" s="18" t="s">
+      <c r="Z1" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="AA1" s="18" t="s">
+      <c r="AA1" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="AB1" s="18" t="s">
+      <c r="AB1" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="AC1" s="18" t="s">
+      <c r="AC1" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="AD1" s="18" t="s">
+      <c r="AD1" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="AE1" s="18" t="s">
+      <c r="AE1" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="AF1" s="18" t="s">
+      <c r="AF1" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="AG1" s="18" t="s">
+      <c r="AG1" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="AH1" s="18" t="s">
+      <c r="AH1" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="AI1" s="18" t="s">
+      <c r="AI1" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="AJ1" s="18" t="s">
+      <c r="AJ1" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="AK1" s="18" t="s">
+      <c r="AK1" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AL1" s="18" t="s">
+      <c r="AL1" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="AM1" s="18" t="s">
+      <c r="AM1" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="AN1" s="18" t="s">
+      <c r="AN1" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="AO1" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="AP1" s="18" t="s">
+      <c r="AO1" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="AP1" s="17" t="s">
         <v>49</v>
       </c>
     </row>
@@ -5361,7 +5370,7 @@
       <c r="A2">
         <v>2007</v>
       </c>
-      <c r="B2" s="17">
+      <c r="B2">
         <v>122</v>
       </c>
       <c r="E2" s="1"/>
@@ -5439,7 +5448,7 @@
       <c r="A3">
         <v>2007</v>
       </c>
-      <c r="B3" s="17">
+      <c r="B3">
         <v>123</v>
       </c>
       <c r="D3" s="1">
@@ -5562,7 +5571,7 @@
       <c r="A4">
         <v>2007</v>
       </c>
-      <c r="B4" s="17">
+      <c r="B4">
         <v>124</v>
       </c>
       <c r="D4" s="1"/>
@@ -5609,7 +5618,7 @@
       <c r="A5">
         <v>2007</v>
       </c>
-      <c r="B5" s="17">
+      <c r="B5">
         <v>127</v>
       </c>
       <c r="D5" s="1">
@@ -5732,7 +5741,7 @@
       <c r="A6">
         <v>2007</v>
       </c>
-      <c r="B6" s="17">
+      <c r="B6">
         <v>130</v>
       </c>
       <c r="D6" s="1">
@@ -5855,7 +5864,7 @@
       <c r="A7">
         <v>2007</v>
       </c>
-      <c r="B7" s="17">
+      <c r="B7">
         <v>155</v>
       </c>
       <c r="D7" s="1">
@@ -5978,7 +5987,7 @@
       <c r="A8">
         <v>2007</v>
       </c>
-      <c r="B8" s="17">
+      <c r="B8">
         <v>169</v>
       </c>
       <c r="D8" s="1"/>
@@ -6049,7 +6058,7 @@
       <c r="A9">
         <v>2007</v>
       </c>
-      <c r="B9" s="17">
+      <c r="B9">
         <v>170</v>
       </c>
       <c r="D9" s="1">
@@ -6108,7 +6117,7 @@
       <c r="A10">
         <v>2007</v>
       </c>
-      <c r="B10" s="17">
+      <c r="B10">
         <v>173</v>
       </c>
       <c r="D10" s="1"/>
@@ -6181,7 +6190,7 @@
       <c r="A11">
         <v>2007</v>
       </c>
-      <c r="B11" s="17">
+      <c r="B11">
         <v>176</v>
       </c>
       <c r="D11" s="1"/>
@@ -6236,7 +6245,7 @@
       <c r="A12">
         <v>2007</v>
       </c>
-      <c r="B12" s="17">
+      <c r="B12">
         <v>179</v>
       </c>
       <c r="D12" s="1">
@@ -6295,7 +6304,7 @@
       <c r="A13">
         <v>2007</v>
       </c>
-      <c r="B13" s="17">
+      <c r="B13">
         <v>180</v>
       </c>
       <c r="D13" s="1"/>
@@ -6366,7 +6375,7 @@
       <c r="A14">
         <v>2007</v>
       </c>
-      <c r="B14" s="17">
+      <c r="B14">
         <v>183</v>
       </c>
       <c r="D14" s="1"/>
@@ -6443,7 +6452,7 @@
       <c r="A15">
         <v>2007</v>
       </c>
-      <c r="B15" s="17">
+      <c r="B15">
         <v>187</v>
       </c>
       <c r="D15" s="1"/>
@@ -6500,7 +6509,7 @@
       <c r="A16">
         <v>2007</v>
       </c>
-      <c r="B16" s="17">
+      <c r="B16">
         <v>190</v>
       </c>
       <c r="D16" s="1"/>
@@ -6571,7 +6580,7 @@
       <c r="A17">
         <v>2007</v>
       </c>
-      <c r="B17" s="17">
+      <c r="B17">
         <v>191</v>
       </c>
       <c r="D17" s="1">
@@ -6624,7 +6633,7 @@
       <c r="A18">
         <v>2007</v>
       </c>
-      <c r="B18" s="17">
+      <c r="B18">
         <v>193</v>
       </c>
       <c r="D18" s="1"/>
@@ -6695,7 +6704,7 @@
       <c r="A19">
         <v>2007</v>
       </c>
-      <c r="B19" s="17">
+      <c r="B19">
         <v>194</v>
       </c>
       <c r="D19" s="1"/>
@@ -6748,7 +6757,7 @@
       <c r="A20">
         <v>2007</v>
       </c>
-      <c r="B20" s="17">
+      <c r="B20">
         <v>201</v>
       </c>
       <c r="D20" s="1"/>
@@ -6811,7 +6820,7 @@
       <c r="A21">
         <v>2007</v>
       </c>
-      <c r="B21" s="17">
+      <c r="B21">
         <v>204</v>
       </c>
       <c r="D21" s="2"/>
@@ -6882,7 +6891,7 @@
       <c r="A22">
         <v>2007</v>
       </c>
-      <c r="B22" s="17">
+      <c r="B22">
         <v>207</v>
       </c>
       <c r="D22" s="1"/>
@@ -6929,7 +6938,7 @@
       <c r="A23">
         <v>2007</v>
       </c>
-      <c r="B23" s="17">
+      <c r="B23">
         <v>208</v>
       </c>
       <c r="D23" s="1"/>
@@ -7006,7 +7015,7 @@
       <c r="A24">
         <v>2007</v>
       </c>
-      <c r="B24" s="17">
+      <c r="B24">
         <v>214</v>
       </c>
       <c r="D24" s="1">
@@ -7059,7 +7068,7 @@
       <c r="A25">
         <v>2007</v>
       </c>
-      <c r="B25" s="17">
+      <c r="B25">
         <v>221</v>
       </c>
       <c r="D25" s="1"/>
@@ -7138,7 +7147,7 @@
       <c r="A26">
         <v>2007</v>
       </c>
-      <c r="B26" s="17">
+      <c r="B26">
         <v>222</v>
       </c>
       <c r="D26" s="1"/>
@@ -7209,7 +7218,7 @@
       <c r="A27">
         <v>2007</v>
       </c>
-      <c r="B27" s="17">
+      <c r="B27">
         <v>225</v>
       </c>
       <c r="D27" s="1"/>
@@ -7262,7 +7271,7 @@
       <c r="A28">
         <v>2007</v>
       </c>
-      <c r="B28" s="17">
+      <c r="B28">
         <v>226</v>
       </c>
       <c r="D28" s="1"/>
@@ -7317,7 +7326,7 @@
       <c r="A29">
         <v>2007</v>
       </c>
-      <c r="B29" s="17">
+      <c r="B29">
         <v>232</v>
       </c>
       <c r="D29" s="1"/>
@@ -7380,7 +7389,7 @@
       <c r="A30">
         <v>2007</v>
       </c>
-      <c r="B30" s="17">
+      <c r="B30">
         <v>233</v>
       </c>
       <c r="D30" s="1">
@@ -7465,7 +7474,7 @@
       <c r="A31">
         <v>2007</v>
       </c>
-      <c r="B31" s="17">
+      <c r="B31">
         <v>234</v>
       </c>
       <c r="D31" s="1"/>
@@ -7512,7 +7521,7 @@
       <c r="A32">
         <v>2007</v>
       </c>
-      <c r="B32" s="17">
+      <c r="B32">
         <v>235</v>
       </c>
       <c r="D32" s="1"/>
@@ -7581,7 +7590,7 @@
       <c r="A33">
         <v>2007</v>
       </c>
-      <c r="B33" s="17">
+      <c r="B33">
         <v>248</v>
       </c>
       <c r="D33" s="1"/>
@@ -7670,7 +7679,7 @@
       <c r="A34">
         <v>2007</v>
       </c>
-      <c r="B34" s="17">
+      <c r="B34">
         <v>249</v>
       </c>
       <c r="D34" s="1">
@@ -7752,7 +7761,2465 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B8598CA-A4FE-4A1E-8BDF-FD66BC2310A1}">
+  <dimension ref="A1:AP26"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="D1" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="E1" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="G1" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="H1" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="I1" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="J1" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="K1" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="L1" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="M1" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="N1" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="O1" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="P1" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q1" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="R1" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="S1" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="T1" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="U1" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="V1" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="W1" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="X1" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="Y1" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="Z1" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA1" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="AB1" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="AC1" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="AD1" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE1" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF1" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="AG1" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="AH1" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="AI1" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AJ1" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="AK1" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL1" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="AM1" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="AN1" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="AO1" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="AP1" s="17" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:42" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B2" s="18">
+        <v>155</v>
+      </c>
+      <c r="F2" s="18">
+        <v>50</v>
+      </c>
+      <c r="G2" s="18">
+        <v>50</v>
+      </c>
+      <c r="H2" s="18">
+        <v>50</v>
+      </c>
+      <c r="I2" s="18">
+        <v>50</v>
+      </c>
+      <c r="J2" s="18">
+        <v>50</v>
+      </c>
+      <c r="K2" s="18">
+        <v>50</v>
+      </c>
+      <c r="L2" s="18">
+        <v>50</v>
+      </c>
+      <c r="M2" s="18">
+        <v>50</v>
+      </c>
+      <c r="N2" s="18">
+        <v>50</v>
+      </c>
+      <c r="O2" s="18">
+        <v>50</v>
+      </c>
+      <c r="P2" s="18">
+        <v>50</v>
+      </c>
+      <c r="Q2" s="18">
+        <v>50</v>
+      </c>
+      <c r="R2" s="18">
+        <v>50</v>
+      </c>
+      <c r="S2" s="18">
+        <v>50</v>
+      </c>
+      <c r="T2" s="18">
+        <v>50</v>
+      </c>
+      <c r="U2" s="18">
+        <v>50</v>
+      </c>
+      <c r="V2" s="18">
+        <v>50</v>
+      </c>
+      <c r="W2" s="18">
+        <v>50</v>
+      </c>
+      <c r="X2" s="18">
+        <v>50</v>
+      </c>
+      <c r="Y2" s="18">
+        <v>50</v>
+      </c>
+      <c r="Z2" s="18">
+        <v>50</v>
+      </c>
+      <c r="AA2" s="18">
+        <v>50</v>
+      </c>
+      <c r="AB2" s="18">
+        <v>50</v>
+      </c>
+      <c r="AC2" s="18">
+        <v>50</v>
+      </c>
+      <c r="AD2" s="18">
+        <v>50</v>
+      </c>
+      <c r="AE2" s="18">
+        <v>50</v>
+      </c>
+      <c r="AF2" s="18">
+        <v>50</v>
+      </c>
+      <c r="AG2" s="18">
+        <v>50</v>
+      </c>
+      <c r="AH2" s="18">
+        <v>50</v>
+      </c>
+      <c r="AI2" s="18">
+        <v>50</v>
+      </c>
+      <c r="AJ2" s="18">
+        <v>50</v>
+      </c>
+      <c r="AM2" s="18">
+        <v>50</v>
+      </c>
+      <c r="AN2" s="18">
+        <v>50</v>
+      </c>
+      <c r="AO2" s="18">
+        <v>50</v>
+      </c>
+      <c r="AP2" s="18">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:42" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B3" s="18">
+        <v>170</v>
+      </c>
+      <c r="D3" s="18">
+        <v>50</v>
+      </c>
+      <c r="AK3" s="18">
+        <v>50</v>
+      </c>
+      <c r="AL3" s="18">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:42" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B4" s="18">
+        <v>179</v>
+      </c>
+      <c r="D4" s="18">
+        <v>50</v>
+      </c>
+      <c r="F4" s="18">
+        <v>50</v>
+      </c>
+      <c r="G4" s="18">
+        <v>50</v>
+      </c>
+      <c r="H4" s="18">
+        <v>50</v>
+      </c>
+      <c r="I4" s="18">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:42" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B5" s="18">
+        <v>180</v>
+      </c>
+      <c r="K5" s="18">
+        <v>50</v>
+      </c>
+      <c r="L5" s="18">
+        <v>50</v>
+      </c>
+      <c r="O5" s="18">
+        <v>50</v>
+      </c>
+      <c r="V5" s="18">
+        <v>50</v>
+      </c>
+      <c r="W5" s="18">
+        <v>50</v>
+      </c>
+      <c r="X5" s="18">
+        <v>50</v>
+      </c>
+      <c r="AA5" s="18">
+        <v>50</v>
+      </c>
+      <c r="AB5" s="18">
+        <v>50</v>
+      </c>
+      <c r="AD5" s="18">
+        <v>50</v>
+      </c>
+      <c r="AF5" s="18">
+        <v>50</v>
+      </c>
+      <c r="AN5" s="18">
+        <v>50</v>
+      </c>
+      <c r="AP5" s="18">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:42" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B6" s="18">
+        <v>183</v>
+      </c>
+      <c r="M6" s="18">
+        <v>50</v>
+      </c>
+      <c r="N6" s="18">
+        <v>50</v>
+      </c>
+      <c r="P6" s="18">
+        <v>50</v>
+      </c>
+      <c r="R6" s="18">
+        <v>50</v>
+      </c>
+      <c r="T6" s="18">
+        <v>50</v>
+      </c>
+      <c r="U6" s="18">
+        <v>50</v>
+      </c>
+      <c r="Z6" s="18">
+        <v>50</v>
+      </c>
+      <c r="AG6" s="18">
+        <v>50</v>
+      </c>
+      <c r="AH6" s="18">
+        <v>50</v>
+      </c>
+      <c r="AI6" s="18">
+        <v>50</v>
+      </c>
+      <c r="AJ6" s="18">
+        <v>50</v>
+      </c>
+      <c r="AK6" s="18">
+        <v>50</v>
+      </c>
+      <c r="AL6" s="18">
+        <v>50</v>
+      </c>
+      <c r="AM6" s="18">
+        <v>50</v>
+      </c>
+      <c r="AO6" s="18">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:42" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B7" s="18">
+        <v>187</v>
+      </c>
+      <c r="Q7" s="18">
+        <v>50</v>
+      </c>
+      <c r="S7" s="18">
+        <v>50</v>
+      </c>
+      <c r="Y7" s="18">
+        <v>50</v>
+      </c>
+      <c r="AC7" s="18">
+        <v>50</v>
+      </c>
+      <c r="AE7" s="18">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:42" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B8" s="18">
+        <v>201</v>
+      </c>
+      <c r="J8" s="18">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:42" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B9" s="18">
+        <v>221</v>
+      </c>
+      <c r="F9" s="18">
+        <v>25</v>
+      </c>
+      <c r="G9" s="18">
+        <v>25</v>
+      </c>
+      <c r="J9" s="18">
+        <v>25</v>
+      </c>
+      <c r="K9" s="18">
+        <v>25</v>
+      </c>
+      <c r="L9" s="18">
+        <v>25</v>
+      </c>
+      <c r="O9" s="18">
+        <v>25</v>
+      </c>
+      <c r="V9" s="18">
+        <v>25</v>
+      </c>
+      <c r="W9" s="18">
+        <v>25</v>
+      </c>
+      <c r="X9" s="18">
+        <v>25</v>
+      </c>
+      <c r="Y9" s="18">
+        <v>25</v>
+      </c>
+      <c r="AA9" s="18">
+        <v>25</v>
+      </c>
+      <c r="AB9" s="18">
+        <v>25</v>
+      </c>
+      <c r="AD9" s="18">
+        <v>25</v>
+      </c>
+      <c r="AF9" s="18">
+        <v>25</v>
+      </c>
+      <c r="AN9" s="18">
+        <v>25</v>
+      </c>
+      <c r="AP9" s="18">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:42" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B10" s="18">
+        <v>222</v>
+      </c>
+      <c r="N10" s="18">
+        <v>25</v>
+      </c>
+      <c r="P10" s="18">
+        <v>25</v>
+      </c>
+      <c r="Q10" s="18">
+        <v>25</v>
+      </c>
+      <c r="R10" s="18">
+        <v>25</v>
+      </c>
+      <c r="S10" s="18">
+        <v>25</v>
+      </c>
+      <c r="T10" s="18">
+        <v>25</v>
+      </c>
+      <c r="AC10" s="18">
+        <v>25</v>
+      </c>
+      <c r="AE10" s="18">
+        <v>25</v>
+      </c>
+      <c r="AG10" s="18">
+        <v>25</v>
+      </c>
+      <c r="AI10" s="18">
+        <v>25</v>
+      </c>
+      <c r="AJ10" s="18">
+        <v>25</v>
+      </c>
+      <c r="AO10" s="18">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:42" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B11" s="18">
+        <v>225</v>
+      </c>
+      <c r="M11" s="18">
+        <v>25</v>
+      </c>
+      <c r="AK11" s="18">
+        <v>25</v>
+      </c>
+      <c r="AL11" s="18">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:42" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B12" s="18">
+        <v>226</v>
+      </c>
+      <c r="U12" s="18">
+        <v>25</v>
+      </c>
+      <c r="Z12" s="18">
+        <v>25</v>
+      </c>
+      <c r="AH12" s="18">
+        <v>25</v>
+      </c>
+      <c r="AM12" s="18">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:42" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:42" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="15" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B15" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="D15" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="G15" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="H15" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="I15" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="J15" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="K15" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="L15" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="M15" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="N15" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="O15" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="P15" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q15" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="R15" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="S15" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="T15" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="U15" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="V15" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="W15" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="X15" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="Y15" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="Z15" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA15" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="AB15" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="AC15" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="AD15" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE15" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF15" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="AG15" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="AH15" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="AI15" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="AJ15" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="AK15" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL15" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="AM15" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="AN15" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="AO15" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="AP15" s="17" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="16" spans="1:42" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B16" s="18">
+        <v>155</v>
+      </c>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19">
+        <f t="shared" ref="D16:AP22" si="0">F2*0.453592/0.404686</f>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="G16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="H16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="I16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="J16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="K16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="L16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="M16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="N16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="O16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="P16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="Q16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="R16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="S16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="T16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="U16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="V16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="W16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="X16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="Y16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="Z16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AA16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AB16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AC16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AD16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AE16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AF16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AG16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AH16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AI16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AJ16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AK16" s="19"/>
+      <c r="AL16" s="19"/>
+      <c r="AM16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AN16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AO16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AP16" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+    </row>
+    <row r="17" spans="1:42" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B17" s="18">
+        <v>170</v>
+      </c>
+      <c r="C17" s="19"/>
+      <c r="D17" s="19">
+        <f t="shared" ref="C17:R26" si="1">D3*0.453592/0.404686</f>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="E17" s="19"/>
+      <c r="F17" s="19"/>
+      <c r="G17" s="19"/>
+      <c r="H17" s="19"/>
+      <c r="I17" s="19"/>
+      <c r="J17" s="19"/>
+      <c r="K17" s="19"/>
+      <c r="L17" s="19"/>
+      <c r="M17" s="19"/>
+      <c r="N17" s="19"/>
+      <c r="O17" s="19"/>
+      <c r="P17" s="19"/>
+      <c r="Q17" s="19"/>
+      <c r="R17" s="19"/>
+      <c r="S17" s="19"/>
+      <c r="T17" s="19"/>
+      <c r="U17" s="19"/>
+      <c r="V17" s="19"/>
+      <c r="W17" s="19"/>
+      <c r="X17" s="19"/>
+      <c r="Y17" s="19"/>
+      <c r="Z17" s="19"/>
+      <c r="AA17" s="19"/>
+      <c r="AB17" s="19"/>
+      <c r="AC17" s="19"/>
+      <c r="AD17" s="19"/>
+      <c r="AE17" s="19"/>
+      <c r="AF17" s="19"/>
+      <c r="AG17" s="19"/>
+      <c r="AH17" s="19"/>
+      <c r="AI17" s="19"/>
+      <c r="AJ17" s="19"/>
+      <c r="AK17" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AL17" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AM17" s="19"/>
+      <c r="AN17" s="19"/>
+      <c r="AO17" s="19"/>
+      <c r="AP17" s="19"/>
+    </row>
+    <row r="18" spans="1:42" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B18" s="18">
+        <v>179</v>
+      </c>
+      <c r="C18" s="19"/>
+      <c r="D18" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="E18" s="19"/>
+      <c r="F18" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="G18" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="H18" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="I18" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="J18" s="19"/>
+      <c r="K18" s="19"/>
+      <c r="L18" s="19"/>
+      <c r="M18" s="19"/>
+      <c r="N18" s="19"/>
+      <c r="O18" s="19"/>
+      <c r="P18" s="19"/>
+      <c r="Q18" s="19"/>
+      <c r="R18" s="19"/>
+      <c r="S18" s="19"/>
+      <c r="T18" s="19"/>
+      <c r="U18" s="19"/>
+      <c r="V18" s="19"/>
+      <c r="W18" s="19"/>
+      <c r="X18" s="19"/>
+      <c r="Y18" s="19"/>
+      <c r="Z18" s="19"/>
+      <c r="AA18" s="19"/>
+      <c r="AB18" s="19"/>
+      <c r="AC18" s="19"/>
+      <c r="AD18" s="19"/>
+      <c r="AE18" s="19"/>
+      <c r="AF18" s="19"/>
+      <c r="AG18" s="19"/>
+      <c r="AH18" s="19"/>
+      <c r="AI18" s="19"/>
+      <c r="AJ18" s="19"/>
+      <c r="AK18" s="19"/>
+      <c r="AL18" s="19"/>
+      <c r="AM18" s="19"/>
+      <c r="AN18" s="19"/>
+      <c r="AO18" s="19"/>
+      <c r="AP18" s="19"/>
+    </row>
+    <row r="19" spans="1:42" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B19" s="18">
+        <v>180</v>
+      </c>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="19"/>
+      <c r="G19" s="19"/>
+      <c r="H19" s="19"/>
+      <c r="I19" s="19"/>
+      <c r="J19" s="19"/>
+      <c r="K19" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="L19" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="M19" s="19"/>
+      <c r="N19" s="19"/>
+      <c r="O19" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="P19" s="19"/>
+      <c r="Q19" s="19"/>
+      <c r="R19" s="19"/>
+      <c r="S19" s="19"/>
+      <c r="T19" s="19"/>
+      <c r="U19" s="19"/>
+      <c r="V19" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="W19" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="X19" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="Y19" s="19"/>
+      <c r="Z19" s="19"/>
+      <c r="AA19" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AB19" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AC19" s="19"/>
+      <c r="AD19" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AE19" s="19"/>
+      <c r="AF19" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AG19" s="19"/>
+      <c r="AH19" s="19"/>
+      <c r="AI19" s="19"/>
+      <c r="AJ19" s="19"/>
+      <c r="AK19" s="19"/>
+      <c r="AL19" s="19"/>
+      <c r="AM19" s="19"/>
+      <c r="AN19" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AO19" s="19"/>
+      <c r="AP19" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+    </row>
+    <row r="20" spans="1:42" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B20" s="18">
+        <v>183</v>
+      </c>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="19"/>
+      <c r="J20" s="19"/>
+      <c r="K20" s="19"/>
+      <c r="L20" s="19"/>
+      <c r="M20" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="N20" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="O20" s="19"/>
+      <c r="P20" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="Q20" s="19"/>
+      <c r="R20" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="S20" s="19"/>
+      <c r="T20" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="U20" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="V20" s="19"/>
+      <c r="W20" s="19"/>
+      <c r="X20" s="19"/>
+      <c r="Y20" s="19"/>
+      <c r="Z20" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AA20" s="19"/>
+      <c r="AB20" s="19"/>
+      <c r="AC20" s="19"/>
+      <c r="AD20" s="19"/>
+      <c r="AE20" s="19"/>
+      <c r="AF20" s="19"/>
+      <c r="AG20" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AH20" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AI20" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AJ20" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AK20" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AL20" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AM20" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AN20" s="19"/>
+      <c r="AO20" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AP20" s="19"/>
+    </row>
+    <row r="21" spans="1:42" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B21" s="18">
+        <v>187</v>
+      </c>
+      <c r="C21" s="19"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="19"/>
+      <c r="G21" s="19"/>
+      <c r="H21" s="19"/>
+      <c r="I21" s="19"/>
+      <c r="J21" s="19"/>
+      <c r="K21" s="19"/>
+      <c r="L21" s="19"/>
+      <c r="M21" s="19"/>
+      <c r="N21" s="19"/>
+      <c r="O21" s="19"/>
+      <c r="P21" s="19"/>
+      <c r="Q21" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="R21" s="19"/>
+      <c r="S21" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="T21" s="19"/>
+      <c r="U21" s="19"/>
+      <c r="V21" s="19"/>
+      <c r="W21" s="19"/>
+      <c r="X21" s="19"/>
+      <c r="Y21" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="Z21" s="19"/>
+      <c r="AA21" s="19"/>
+      <c r="AB21" s="19"/>
+      <c r="AC21" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AD21" s="19"/>
+      <c r="AE21" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AF21" s="19"/>
+      <c r="AG21" s="19"/>
+      <c r="AH21" s="19"/>
+      <c r="AI21" s="19"/>
+      <c r="AJ21" s="19"/>
+      <c r="AK21" s="19"/>
+      <c r="AL21" s="19"/>
+      <c r="AM21" s="19"/>
+      <c r="AN21" s="19"/>
+      <c r="AO21" s="19"/>
+      <c r="AP21" s="19"/>
+    </row>
+    <row r="22" spans="1:42" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B22" s="18">
+        <v>201</v>
+      </c>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="19"/>
+      <c r="G22" s="19"/>
+      <c r="H22" s="19"/>
+      <c r="I22" s="19"/>
+      <c r="J22" s="19">
+        <f t="shared" si="0"/>
+        <v>56.042462551212544</v>
+      </c>
+      <c r="K22" s="19"/>
+      <c r="L22" s="19"/>
+      <c r="M22" s="19"/>
+      <c r="N22" s="19"/>
+      <c r="O22" s="19"/>
+      <c r="P22" s="19"/>
+      <c r="Q22" s="19"/>
+      <c r="R22" s="19"/>
+      <c r="S22" s="19"/>
+      <c r="T22" s="19"/>
+      <c r="U22" s="19"/>
+      <c r="V22" s="19"/>
+      <c r="W22" s="19"/>
+      <c r="X22" s="19"/>
+      <c r="Y22" s="19"/>
+      <c r="Z22" s="19"/>
+      <c r="AA22" s="19"/>
+      <c r="AB22" s="19"/>
+      <c r="AC22" s="19"/>
+      <c r="AD22" s="19"/>
+      <c r="AE22" s="19"/>
+      <c r="AF22" s="19"/>
+      <c r="AG22" s="19"/>
+      <c r="AH22" s="19"/>
+      <c r="AI22" s="19"/>
+      <c r="AJ22" s="19"/>
+      <c r="AK22" s="19"/>
+      <c r="AL22" s="19"/>
+      <c r="AM22" s="19"/>
+      <c r="AN22" s="19"/>
+      <c r="AO22" s="19"/>
+      <c r="AP22" s="19"/>
+    </row>
+    <row r="23" spans="1:42" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B23" s="18">
+        <v>221</v>
+      </c>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19">
+        <f t="shared" ref="D22:AP26" si="2">F9*0.453592/0.404686</f>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="G23" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="H23" s="19"/>
+      <c r="I23" s="19"/>
+      <c r="J23" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="K23" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="L23" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="M23" s="19"/>
+      <c r="N23" s="19"/>
+      <c r="O23" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="P23" s="19"/>
+      <c r="Q23" s="19"/>
+      <c r="R23" s="19"/>
+      <c r="S23" s="19"/>
+      <c r="T23" s="19"/>
+      <c r="U23" s="19"/>
+      <c r="V23" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="W23" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="X23" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="Y23" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="Z23" s="19"/>
+      <c r="AA23" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AB23" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AC23" s="19"/>
+      <c r="AD23" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AE23" s="19"/>
+      <c r="AF23" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AG23" s="19"/>
+      <c r="AH23" s="19"/>
+      <c r="AI23" s="19"/>
+      <c r="AJ23" s="19"/>
+      <c r="AK23" s="19"/>
+      <c r="AL23" s="19"/>
+      <c r="AM23" s="19"/>
+      <c r="AN23" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AO23" s="19"/>
+      <c r="AP23" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+    </row>
+    <row r="24" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A24" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B24" s="18">
+        <v>222</v>
+      </c>
+      <c r="C24" s="19"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="19"/>
+      <c r="G24" s="19"/>
+      <c r="H24" s="19"/>
+      <c r="I24" s="19"/>
+      <c r="J24" s="19"/>
+      <c r="K24" s="19"/>
+      <c r="L24" s="19"/>
+      <c r="M24" s="19"/>
+      <c r="N24" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="O24" s="19"/>
+      <c r="P24" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="Q24" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="R24" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="S24" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="T24" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="U24" s="19"/>
+      <c r="V24" s="19"/>
+      <c r="W24" s="19"/>
+      <c r="X24" s="19"/>
+      <c r="Y24" s="19"/>
+      <c r="Z24" s="19"/>
+      <c r="AA24" s="19"/>
+      <c r="AB24" s="19"/>
+      <c r="AC24" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AD24" s="19"/>
+      <c r="AE24" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AF24" s="19"/>
+      <c r="AG24" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AH24" s="19"/>
+      <c r="AI24" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AJ24" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AK24" s="19"/>
+      <c r="AL24" s="19"/>
+      <c r="AM24" s="19"/>
+      <c r="AN24" s="19"/>
+      <c r="AO24" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AP24" s="19"/>
+    </row>
+    <row r="25" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A25" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B25" s="18">
+        <v>225</v>
+      </c>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="19"/>
+      <c r="G25" s="19"/>
+      <c r="H25" s="19"/>
+      <c r="I25" s="19"/>
+      <c r="J25" s="19"/>
+      <c r="K25" s="19"/>
+      <c r="L25" s="19"/>
+      <c r="M25" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="N25" s="19"/>
+      <c r="O25" s="19"/>
+      <c r="P25" s="19"/>
+      <c r="Q25" s="19"/>
+      <c r="R25" s="19"/>
+      <c r="S25" s="19"/>
+      <c r="T25" s="19"/>
+      <c r="U25" s="19"/>
+      <c r="V25" s="19"/>
+      <c r="W25" s="19"/>
+      <c r="X25" s="19"/>
+      <c r="Y25" s="19"/>
+      <c r="Z25" s="19"/>
+      <c r="AA25" s="19"/>
+      <c r="AB25" s="19"/>
+      <c r="AC25" s="19"/>
+      <c r="AD25" s="19"/>
+      <c r="AE25" s="19"/>
+      <c r="AF25" s="19"/>
+      <c r="AG25" s="19"/>
+      <c r="AH25" s="19"/>
+      <c r="AI25" s="19"/>
+      <c r="AJ25" s="19"/>
+      <c r="AK25" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AL25" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AM25" s="19"/>
+      <c r="AN25" s="19"/>
+      <c r="AO25" s="19"/>
+      <c r="AP25" s="19"/>
+    </row>
+    <row r="26" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A26" s="18">
+        <v>2007</v>
+      </c>
+      <c r="B26" s="18">
+        <v>226</v>
+      </c>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
+      <c r="G26" s="19"/>
+      <c r="H26" s="19"/>
+      <c r="I26" s="19"/>
+      <c r="J26" s="19"/>
+      <c r="K26" s="19"/>
+      <c r="L26" s="19"/>
+      <c r="M26" s="19"/>
+      <c r="N26" s="19"/>
+      <c r="O26" s="19"/>
+      <c r="P26" s="19"/>
+      <c r="Q26" s="19"/>
+      <c r="R26" s="19"/>
+      <c r="S26" s="19"/>
+      <c r="T26" s="19"/>
+      <c r="U26" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="V26" s="19"/>
+      <c r="W26" s="19"/>
+      <c r="X26" s="19"/>
+      <c r="Y26" s="19"/>
+      <c r="Z26" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AA26" s="19"/>
+      <c r="AB26" s="19"/>
+      <c r="AC26" s="19"/>
+      <c r="AD26" s="19"/>
+      <c r="AE26" s="19"/>
+      <c r="AF26" s="19"/>
+      <c r="AG26" s="19"/>
+      <c r="AH26" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AI26" s="19"/>
+      <c r="AJ26" s="19"/>
+      <c r="AK26" s="19"/>
+      <c r="AL26" s="19"/>
+      <c r="AM26" s="19">
+        <f t="shared" si="2"/>
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AN26" s="19"/>
+      <c r="AO26" s="19"/>
+      <c r="AP26" s="19"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FAAA557-8B6D-45D6-BA08-859BEB94955E}">
+  <dimension ref="A1:AP12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1" t="s">
+        <v>84</v>
+      </c>
+      <c r="G1" t="s">
+        <v>85</v>
+      </c>
+      <c r="H1" t="s">
+        <v>86</v>
+      </c>
+      <c r="I1" t="s">
+        <v>87</v>
+      </c>
+      <c r="J1" t="s">
+        <v>88</v>
+      </c>
+      <c r="K1" t="s">
+        <v>65</v>
+      </c>
+      <c r="L1" t="s">
+        <v>66</v>
+      </c>
+      <c r="M1" t="s">
+        <v>67</v>
+      </c>
+      <c r="N1" t="s">
+        <v>68</v>
+      </c>
+      <c r="O1" t="s">
+        <v>69</v>
+      </c>
+      <c r="P1" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>71</v>
+      </c>
+      <c r="R1" t="s">
+        <v>72</v>
+      </c>
+      <c r="S1" t="s">
+        <v>73</v>
+      </c>
+      <c r="T1" t="s">
+        <v>74</v>
+      </c>
+      <c r="U1" t="s">
+        <v>75</v>
+      </c>
+      <c r="V1" t="s">
+        <v>76</v>
+      </c>
+      <c r="W1" t="s">
+        <v>77</v>
+      </c>
+      <c r="X1" t="s">
+        <v>78</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>79</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>64</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>63</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>62</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>61</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>59</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>58</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>57</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>56</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>55</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>53</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>52</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>51</v>
+      </c>
+      <c r="AO1" t="s">
+        <v>50</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2007</v>
+      </c>
+      <c r="B2">
+        <v>155</v>
+      </c>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="G2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="H2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="I2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="J2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="K2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="L2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="M2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="N2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="O2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="P2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="Q2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="R2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="S2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="T2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="U2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="V2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="W2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="X2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="Y2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="Z2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AA2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AB2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AC2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AD2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AE2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AF2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AG2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AH2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AI2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AJ2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AK2" s="20"/>
+      <c r="AL2" s="20"/>
+      <c r="AM2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AN2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AO2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AP2" s="20">
+        <v>56.042462551212544</v>
+      </c>
+    </row>
+    <row r="3" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2007</v>
+      </c>
+      <c r="B3">
+        <v>170</v>
+      </c>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
+      <c r="L3" s="20"/>
+      <c r="M3" s="20"/>
+      <c r="N3" s="20"/>
+      <c r="O3" s="20"/>
+      <c r="P3" s="20"/>
+      <c r="Q3" s="20"/>
+      <c r="R3" s="20"/>
+      <c r="S3" s="20"/>
+      <c r="T3" s="20"/>
+      <c r="U3" s="20"/>
+      <c r="V3" s="20"/>
+      <c r="W3" s="20"/>
+      <c r="X3" s="20"/>
+      <c r="Y3" s="20"/>
+      <c r="Z3" s="20"/>
+      <c r="AA3" s="20"/>
+      <c r="AB3" s="20"/>
+      <c r="AC3" s="20"/>
+      <c r="AD3" s="20"/>
+      <c r="AE3" s="20"/>
+      <c r="AF3" s="20"/>
+      <c r="AG3" s="20"/>
+      <c r="AH3" s="20"/>
+      <c r="AI3" s="20"/>
+      <c r="AJ3" s="20"/>
+      <c r="AK3" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AL3" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AM3" s="20"/>
+      <c r="AN3" s="20"/>
+      <c r="AO3" s="20"/>
+      <c r="AP3" s="20"/>
+    </row>
+    <row r="4" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2007</v>
+      </c>
+      <c r="B4">
+        <v>179</v>
+      </c>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="G4" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="H4" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="I4" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="J4" s="20"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="20"/>
+      <c r="M4" s="20"/>
+      <c r="N4" s="20"/>
+      <c r="O4" s="20"/>
+      <c r="P4" s="20"/>
+      <c r="Q4" s="20"/>
+      <c r="R4" s="20"/>
+      <c r="S4" s="20"/>
+      <c r="T4" s="20"/>
+      <c r="U4" s="20"/>
+      <c r="V4" s="20"/>
+      <c r="W4" s="20"/>
+      <c r="X4" s="20"/>
+      <c r="Y4" s="20"/>
+      <c r="Z4" s="20"/>
+      <c r="AA4" s="20"/>
+      <c r="AB4" s="20"/>
+      <c r="AC4" s="20"/>
+      <c r="AD4" s="20"/>
+      <c r="AE4" s="20"/>
+      <c r="AF4" s="20"/>
+      <c r="AG4" s="20"/>
+      <c r="AH4" s="20"/>
+      <c r="AI4" s="20"/>
+      <c r="AJ4" s="20"/>
+      <c r="AK4" s="20"/>
+      <c r="AL4" s="20"/>
+      <c r="AM4" s="20"/>
+      <c r="AN4" s="20"/>
+      <c r="AO4" s="20"/>
+      <c r="AP4" s="20"/>
+    </row>
+    <row r="5" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2007</v>
+      </c>
+      <c r="B5">
+        <v>180</v>
+      </c>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20"/>
+      <c r="H5" s="20"/>
+      <c r="I5" s="20"/>
+      <c r="J5" s="20"/>
+      <c r="K5" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="L5" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="M5" s="20"/>
+      <c r="N5" s="20"/>
+      <c r="O5" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="P5" s="20"/>
+      <c r="Q5" s="20"/>
+      <c r="R5" s="20"/>
+      <c r="S5" s="20"/>
+      <c r="T5" s="20"/>
+      <c r="U5" s="20"/>
+      <c r="V5" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="W5" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="X5" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="Y5" s="20"/>
+      <c r="Z5" s="20"/>
+      <c r="AA5" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AB5" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AC5" s="20"/>
+      <c r="AD5" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AE5" s="20"/>
+      <c r="AF5" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AG5" s="20"/>
+      <c r="AH5" s="20"/>
+      <c r="AI5" s="20"/>
+      <c r="AJ5" s="20"/>
+      <c r="AK5" s="20"/>
+      <c r="AL5" s="20"/>
+      <c r="AM5" s="20"/>
+      <c r="AN5" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AO5" s="20"/>
+      <c r="AP5" s="20">
+        <v>56.042462551212544</v>
+      </c>
+    </row>
+    <row r="6" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2007</v>
+      </c>
+      <c r="B6">
+        <v>183</v>
+      </c>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="20"/>
+      <c r="J6" s="20"/>
+      <c r="K6" s="20"/>
+      <c r="L6" s="20"/>
+      <c r="M6" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="N6" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="O6" s="20"/>
+      <c r="P6" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="Q6" s="20"/>
+      <c r="R6" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="S6" s="20"/>
+      <c r="T6" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="U6" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="V6" s="20"/>
+      <c r="W6" s="20"/>
+      <c r="X6" s="20"/>
+      <c r="Y6" s="20"/>
+      <c r="Z6" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AA6" s="20"/>
+      <c r="AB6" s="20"/>
+      <c r="AC6" s="20"/>
+      <c r="AD6" s="20"/>
+      <c r="AE6" s="20"/>
+      <c r="AF6" s="20"/>
+      <c r="AG6" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AH6" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AI6" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AJ6" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AK6" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AL6" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AM6" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AN6" s="20"/>
+      <c r="AO6" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AP6" s="20"/>
+    </row>
+    <row r="7" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2007</v>
+      </c>
+      <c r="B7">
+        <v>187</v>
+      </c>
+      <c r="C7" s="20"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="20"/>
+      <c r="I7" s="20"/>
+      <c r="J7" s="20"/>
+      <c r="K7" s="20"/>
+      <c r="L7" s="20"/>
+      <c r="M7" s="20"/>
+      <c r="N7" s="20"/>
+      <c r="O7" s="20"/>
+      <c r="P7" s="20"/>
+      <c r="Q7" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="R7" s="20"/>
+      <c r="S7" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="T7" s="20"/>
+      <c r="U7" s="20"/>
+      <c r="V7" s="20"/>
+      <c r="W7" s="20"/>
+      <c r="X7" s="20"/>
+      <c r="Y7" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="Z7" s="20"/>
+      <c r="AA7" s="20"/>
+      <c r="AB7" s="20"/>
+      <c r="AC7" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AD7" s="20"/>
+      <c r="AE7" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="AF7" s="20"/>
+      <c r="AG7" s="20"/>
+      <c r="AH7" s="20"/>
+      <c r="AI7" s="20"/>
+      <c r="AJ7" s="20"/>
+      <c r="AK7" s="20"/>
+      <c r="AL7" s="20"/>
+      <c r="AM7" s="20"/>
+      <c r="AN7" s="20"/>
+      <c r="AO7" s="20"/>
+      <c r="AP7" s="20"/>
+    </row>
+    <row r="8" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>2007</v>
+      </c>
+      <c r="B8">
+        <v>201</v>
+      </c>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="20"/>
+      <c r="J8" s="20">
+        <v>56.042462551212544</v>
+      </c>
+      <c r="K8" s="20"/>
+      <c r="L8" s="20"/>
+      <c r="M8" s="20"/>
+      <c r="N8" s="20"/>
+      <c r="O8" s="20"/>
+      <c r="P8" s="20"/>
+      <c r="Q8" s="20"/>
+      <c r="R8" s="20"/>
+      <c r="S8" s="20"/>
+      <c r="T8" s="20"/>
+      <c r="U8" s="20"/>
+      <c r="V8" s="20"/>
+      <c r="W8" s="20"/>
+      <c r="X8" s="20"/>
+      <c r="Y8" s="20"/>
+      <c r="Z8" s="20"/>
+      <c r="AA8" s="20"/>
+      <c r="AB8" s="20"/>
+      <c r="AC8" s="20"/>
+      <c r="AD8" s="20"/>
+      <c r="AE8" s="20"/>
+      <c r="AF8" s="20"/>
+      <c r="AG8" s="20"/>
+      <c r="AH8" s="20"/>
+      <c r="AI8" s="20"/>
+      <c r="AJ8" s="20"/>
+      <c r="AK8" s="20"/>
+      <c r="AL8" s="20"/>
+      <c r="AM8" s="20"/>
+      <c r="AN8" s="20"/>
+      <c r="AO8" s="20"/>
+      <c r="AP8" s="20"/>
+    </row>
+    <row r="9" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>2007</v>
+      </c>
+      <c r="B9">
+        <v>221</v>
+      </c>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="G9" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="K9" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="L9" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="M9" s="20"/>
+      <c r="N9" s="20"/>
+      <c r="O9" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="P9" s="20"/>
+      <c r="Q9" s="20"/>
+      <c r="R9" s="20"/>
+      <c r="S9" s="20"/>
+      <c r="T9" s="20"/>
+      <c r="U9" s="20"/>
+      <c r="V9" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="W9" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="X9" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="Y9" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="Z9" s="20"/>
+      <c r="AA9" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AB9" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AC9" s="20"/>
+      <c r="AD9" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AE9" s="20"/>
+      <c r="AF9" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AG9" s="20"/>
+      <c r="AH9" s="20"/>
+      <c r="AI9" s="20"/>
+      <c r="AJ9" s="20"/>
+      <c r="AK9" s="20"/>
+      <c r="AL9" s="20"/>
+      <c r="AM9" s="20"/>
+      <c r="AN9" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AO9" s="20"/>
+      <c r="AP9" s="20">
+        <v>28.021231275606272</v>
+      </c>
+    </row>
+    <row r="10" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>2007</v>
+      </c>
+      <c r="B10">
+        <v>222</v>
+      </c>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="20"/>
+      <c r="H10" s="20"/>
+      <c r="I10" s="20"/>
+      <c r="J10" s="20"/>
+      <c r="K10" s="20"/>
+      <c r="L10" s="20"/>
+      <c r="M10" s="20"/>
+      <c r="N10" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="O10" s="20"/>
+      <c r="P10" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="Q10" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="R10" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="S10" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="T10" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="U10" s="20"/>
+      <c r="V10" s="20"/>
+      <c r="W10" s="20"/>
+      <c r="X10" s="20"/>
+      <c r="Y10" s="20"/>
+      <c r="Z10" s="20"/>
+      <c r="AA10" s="20"/>
+      <c r="AB10" s="20"/>
+      <c r="AC10" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AD10" s="20"/>
+      <c r="AE10" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AF10" s="20"/>
+      <c r="AG10" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AH10" s="20"/>
+      <c r="AI10" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AJ10" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AK10" s="20"/>
+      <c r="AL10" s="20"/>
+      <c r="AM10" s="20"/>
+      <c r="AN10" s="20"/>
+      <c r="AO10" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AP10" s="20"/>
+    </row>
+    <row r="11" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>2007</v>
+      </c>
+      <c r="B11">
+        <v>225</v>
+      </c>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="20"/>
+      <c r="G11" s="20"/>
+      <c r="H11" s="20"/>
+      <c r="I11" s="20"/>
+      <c r="J11" s="20"/>
+      <c r="K11" s="20"/>
+      <c r="L11" s="20"/>
+      <c r="M11" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="N11" s="20"/>
+      <c r="O11" s="20"/>
+      <c r="P11" s="20"/>
+      <c r="Q11" s="20"/>
+      <c r="R11" s="20"/>
+      <c r="S11" s="20"/>
+      <c r="T11" s="20"/>
+      <c r="U11" s="20"/>
+      <c r="V11" s="20"/>
+      <c r="W11" s="20"/>
+      <c r="X11" s="20"/>
+      <c r="Y11" s="20"/>
+      <c r="Z11" s="20"/>
+      <c r="AA11" s="20"/>
+      <c r="AB11" s="20"/>
+      <c r="AC11" s="20"/>
+      <c r="AD11" s="20"/>
+      <c r="AE11" s="20"/>
+      <c r="AF11" s="20"/>
+      <c r="AG11" s="20"/>
+      <c r="AH11" s="20"/>
+      <c r="AI11" s="20"/>
+      <c r="AJ11" s="20"/>
+      <c r="AK11" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AL11" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AM11" s="20"/>
+      <c r="AN11" s="20"/>
+      <c r="AO11" s="20"/>
+      <c r="AP11" s="20"/>
+    </row>
+    <row r="12" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>2007</v>
+      </c>
+      <c r="B12">
+        <v>226</v>
+      </c>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
+      <c r="H12" s="20"/>
+      <c r="I12" s="20"/>
+      <c r="J12" s="20"/>
+      <c r="K12" s="20"/>
+      <c r="L12" s="20"/>
+      <c r="M12" s="20"/>
+      <c r="N12" s="20"/>
+      <c r="O12" s="20"/>
+      <c r="P12" s="20"/>
+      <c r="Q12" s="20"/>
+      <c r="R12" s="20"/>
+      <c r="S12" s="20"/>
+      <c r="T12" s="20"/>
+      <c r="U12" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="V12" s="20"/>
+      <c r="W12" s="20"/>
+      <c r="X12" s="20"/>
+      <c r="Y12" s="20"/>
+      <c r="Z12" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AA12" s="20"/>
+      <c r="AB12" s="20"/>
+      <c r="AC12" s="20"/>
+      <c r="AD12" s="20"/>
+      <c r="AE12" s="20"/>
+      <c r="AF12" s="20"/>
+      <c r="AG12" s="20"/>
+      <c r="AH12" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AI12" s="20"/>
+      <c r="AJ12" s="20"/>
+      <c r="AK12" s="20"/>
+      <c r="AL12" s="20"/>
+      <c r="AM12" s="20">
+        <v>28.021231275606272</v>
+      </c>
+      <c r="AN12" s="20"/>
+      <c r="AO12" s="20"/>
+      <c r="AP12" s="20"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001E2F74E811AAA4409A164A292B7ABC74" ma:contentTypeVersion="5" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a274884ad72c80bb9b486423286f1f97">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="728ae82c-3d1b-45f0-8d67-959bce25b5b0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0920719d7b65f5660acd9896835e0dd0" ns3:_="">
     <xsd:import namespace="728ae82c-3d1b-45f0-8d67-959bce25b5b0"/>
@@ -7902,22 +10369,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F50124F-CD4B-4CD9-87F6-3B7F049F2596}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="728ae82c-3d1b-45f0-8d67-959bce25b5b0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B35975F-61E2-43FE-BC08-9ABF3DB94E42}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9ACF685-1BDC-4694-A361-04695E4721A8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7933,28 +10409,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B35975F-61E2-43FE-BC08-9ABF3DB94E42}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F50124F-CD4B-4CD9-87F6-3B7F049F2596}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="728ae82c-3d1b-45f0-8d67-959bce25b5b0"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Finished adding 2003 FISE data
</commit_message>
<xml_diff>
--- a/Data/2007_F111_CO_ISM/2007_F111_CO_ISM_Management.xlsx
+++ b/Data/2007_F111_CO_ISM/2007_F111_CO_ISM_Management.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mnt\Data1\USDA-ALARC\GIS\PDI project\cottondata\Data\2007_F111_CO_ISM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B555EA4D-350A-4417-8E29-882206A2A58E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1526CDAD-CD9F-4BE5-8160-F8E94EBB84F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16470" yWindow="-25965" windowWidth="17865" windowHeight="22530" activeTab="4" xr2:uid="{118525E0-BC31-4C3F-8132-452FA3C5B73C}"/>
+    <workbookView xWindow="-1665" yWindow="-28410" windowWidth="18015" windowHeight="20910" xr2:uid="{118525E0-BC31-4C3F-8132-452FA3C5B73C}"/>
   </bookViews>
   <sheets>
     <sheet name="Irrigation" sheetId="3" r:id="rId1"/>
-    <sheet name="Timeline" sheetId="2" r:id="rId2"/>
+    <sheet name="Timeline" sheetId="7" r:id="rId2"/>
     <sheet name="IrrigationDF" sheetId="1" r:id="rId3"/>
     <sheet name="Fertilizer" sheetId="4" r:id="rId4"/>
     <sheet name="FertilizerDF" sheetId="5" r:id="rId5"/>
@@ -443,6 +443,7 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -454,11 +455,13 @@
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -5225,7 +5228,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD7B9310-504B-4ACD-8CEA-790DF0711A02}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE3A6086-E3EE-4C87-8DCF-64EEFE02944C}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -8611,7 +8614,7 @@
       </c>
       <c r="C17" s="19"/>
       <c r="D17" s="19">
-        <f t="shared" ref="C17:R26" si="1">D3*0.453592/0.404686</f>
+        <f t="shared" ref="D17" si="1">D3*0.453592/0.404686</f>
         <v>56.042462551212544</v>
       </c>
       <c r="E17" s="19"/>
@@ -9024,7 +9027,7 @@
       <c r="D23" s="19"/>
       <c r="E23" s="19"/>
       <c r="F23" s="19">
-        <f t="shared" ref="D22:AP26" si="2">F9*0.453592/0.404686</f>
+        <f t="shared" ref="F23:AP26" si="2">F9*0.453592/0.404686</f>
         <v>28.021231275606272</v>
       </c>
       <c r="G23" s="19">

</xml_diff>